<commit_message>
Build 83: the order carried through
- The six-to-ten printer test is one table read across: builders, homes a
  year, Titans, against ICON's six to ten
- Field view from nearest to farthest; ICON's record in a buyer's order
- Limits open with Scope; five headlines that did not serve the message reverted
- Cover cards cut at a word, not mid-word; channel line not repeated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NR5Yz6eHWvRJ2ZJ71kQKG5
</commit_message>
<xml_diff>
--- a/docs/DFW_Rolodex.xlsx
+++ b/docs/DFW_Rolodex.xlsx
@@ -10940,7 +10940,7 @@
       </c>
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>Trussway had six plants and 1,000 staff when bought, 2022</t>
+          <t>Fort Worth truss and wall-panel plant, formerly Trussway</t>
         </is>
       </c>
       <c r="I87" s="8" t="inlineStr">
@@ -11053,7 +11053,7 @@
       </c>
       <c r="H88" s="12" t="inlineStr">
         <is>
-          <t>Serving the Texas market since 1988</t>
+          <t>Cedar Park precast plant, named North Texas consultant</t>
         </is>
       </c>
       <c r="I88" s="14" t="inlineStr">
@@ -11174,7 +11174,7 @@
       </c>
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>Serving the Texas market since 1988</t>
+          <t>Cedar Park precast plant, named North Texas consultant</t>
         </is>
       </c>
       <c r="I89" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Subscription links stay, listed after the free ones
A paywalled link is no longer removed. The 12 taken off in Build 84 are
back, all 34 carry the Subscription label, and every Sources, press and news
list, and the ICON record's links, put free links first. A precedent row or a
contact takes the free page and the locked one follows it. The workbook's
latest press item is the newest free one. emit.py stops the build if a list
puts a subscription link first.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NR5Yz6eHWvRJ2ZJ71kQKG5
</commit_message>
<xml_diff>
--- a/docs/DFW_Rolodex.xlsx
+++ b/docs/DFW_Rolodex.xlsx
@@ -5268,7 +5268,11 @@
         </is>
       </c>
       <c r="X41" s="6" t="inlineStr"/>
-      <c r="Y41" s="6" t="inlineStr"/>
+      <c r="Y41" s="6" t="inlineStr">
+        <is>
+          <t>2023-07-07 Dallas Morning News. Chicago builder that left D-FW returns to area, takes 1,500 home sites  https://www.dallasnews.com/business/real-estate/2023/07/07/chicago-builder-that-left-d-fw-returns-to-area-takes-1500-home-sites/</t>
+        </is>
+      </c>
       <c r="Z41" s="6" t="inlineStr"/>
       <c r="AA41" s="6" t="inlineStr"/>
       <c r="AB41" s="6" t="inlineStr"/>
@@ -6393,7 +6397,11 @@
           <t>https://www.firsttexashomes.com/about/</t>
         </is>
       </c>
-      <c r="Y50" s="12" t="inlineStr"/>
+      <c r="Y50" s="12" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z50" s="12" t="inlineStr">
         <is>
           <t>(214) 613-3400</t>
@@ -18623,7 +18631,11 @@
           <t>https://www.businesswire.com/news/home/20250821913928/en/PulteGroup-Promotes-Scott-Bryson-to-Dallas-Division-President</t>
         </is>
       </c>
-      <c r="Y148" s="12" t="inlineStr"/>
+      <c r="Y148" s="12" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z148" s="12" t="inlineStr">
         <is>
           <t>(972) 200-3727</t>
@@ -18752,7 +18764,11 @@
           <t>https://www.davidweekleyhomes.com/about-us</t>
         </is>
       </c>
-      <c r="Y149" s="6" t="inlineStr"/>
+      <c r="Y149" s="6" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z149" s="6" t="inlineStr">
         <is>
           <t>(877) 933-5539</t>
@@ -18877,7 +18893,11 @@
           <t>https://www.davidweekleyhomes.com/about-us</t>
         </is>
       </c>
-      <c r="Y150" s="12" t="inlineStr"/>
+      <c r="Y150" s="12" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z150" s="12" t="inlineStr">
         <is>
           <t>(877) 933-5539</t>
@@ -19006,7 +19026,11 @@
           <t>https://www.davidweekleyhomes.com/about-us</t>
         </is>
       </c>
-      <c r="Y151" s="6" t="inlineStr"/>
+      <c r="Y151" s="6" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z151" s="6" t="inlineStr">
         <is>
           <t>(877) 933-5539</t>
@@ -19131,7 +19155,11 @@
           <t>https://www.davidweekleyhomes.com/about-us</t>
         </is>
       </c>
-      <c r="Y152" s="12" t="inlineStr"/>
+      <c r="Y152" s="12" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z152" s="12" t="inlineStr">
         <is>
           <t>(877) 933-5539</t>
@@ -19772,7 +19800,11 @@
           <t>https://investors.meritagehomes.com/company-information/management-team</t>
         </is>
       </c>
-      <c r="Y157" s="6" t="inlineStr"/>
+      <c r="Y157" s="6" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z157" s="6" t="inlineStr">
         <is>
           <t>(469) 487-7973</t>
@@ -19901,7 +19933,11 @@
           <t>https://investors.meritagehomes.com/company-information/management-team</t>
         </is>
       </c>
-      <c r="Y158" s="12" t="inlineStr"/>
+      <c r="Y158" s="12" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z158" s="12" t="inlineStr">
         <is>
           <t>(469) 487-7973</t>
@@ -20030,7 +20066,11 @@
           <t>https://investors.meritagehomes.com/company-information/management-team</t>
         </is>
       </c>
-      <c r="Y159" s="6" t="inlineStr"/>
+      <c r="Y159" s="6" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z159" s="6" t="inlineStr">
         <is>
           <t>(469) 487-7973</t>
@@ -20159,7 +20199,11 @@
           <t>https://www.ashtonwoods.com/corporate-info</t>
         </is>
       </c>
-      <c r="Y160" s="12" t="inlineStr"/>
+      <c r="Y160" s="12" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z160" s="12" t="inlineStr">
         <is>
           <t>(770) 998-9663</t>
@@ -20292,7 +20336,11 @@
           <t>https://www.ashtonwoods.com/corporate-info</t>
         </is>
       </c>
-      <c r="Y161" s="6" t="inlineStr"/>
+      <c r="Y161" s="6" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z161" s="6" t="inlineStr">
         <is>
           <t>(770) 998-9663</t>
@@ -20425,7 +20473,11 @@
           <t>https://www.ashtonwoods.com/corporate-info</t>
         </is>
       </c>
-      <c r="Y162" s="12" t="inlineStr"/>
+      <c r="Y162" s="12" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z162" s="12" t="inlineStr">
         <is>
           <t>(770) 998-9663</t>
@@ -20554,7 +20606,11 @@
           <t>https://www.ashtonwoods.com/corporate-info</t>
         </is>
       </c>
-      <c r="Y163" s="6" t="inlineStr"/>
+      <c r="Y163" s="6" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z163" s="6" t="inlineStr">
         <is>
           <t>(770) 998-9663</t>
@@ -20679,7 +20735,11 @@
           <t>https://www.perryhomes.com/about-perry-homes</t>
         </is>
       </c>
-      <c r="Y164" s="12" t="inlineStr"/>
+      <c r="Y164" s="12" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z164" s="12" t="inlineStr">
         <is>
           <t>(800) 247-3779</t>
@@ -20808,7 +20868,11 @@
           <t>https://www.perryhomes.com/about-perry-homes</t>
         </is>
       </c>
-      <c r="Y165" s="6" t="inlineStr"/>
+      <c r="Y165" s="6" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z165" s="6" t="inlineStr">
         <is>
           <t>(800) 247-3779</t>
@@ -21320,7 +21384,11 @@
           <t>https://greenbrickpartners.com/leadership/</t>
         </is>
       </c>
-      <c r="Y169" s="6" t="inlineStr"/>
+      <c r="Y169" s="6" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z169" s="6" t="inlineStr">
         <is>
           <t>(469) 573-6721</t>
@@ -21449,7 +21517,11 @@
           <t>https://greenbrickpartners.com/leadership/</t>
         </is>
       </c>
-      <c r="Y170" s="12" t="inlineStr"/>
+      <c r="Y170" s="12" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z170" s="12" t="inlineStr">
         <is>
           <t>(469) 573-6721</t>
@@ -21574,7 +21646,11 @@
           <t>https://greenbrickpartners.com/leadership/</t>
         </is>
       </c>
-      <c r="Y171" s="6" t="inlineStr"/>
+      <c r="Y171" s="6" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z171" s="6" t="inlineStr">
         <is>
           <t>(469) 573-6721</t>
@@ -21703,7 +21779,11 @@
           <t>https://greenbrickpartners.com/leadership/</t>
         </is>
       </c>
-      <c r="Y172" s="12" t="inlineStr"/>
+      <c r="Y172" s="12" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z172" s="12" t="inlineStr">
         <is>
           <t>(469) 573-6721</t>
@@ -27812,7 +27892,11 @@
           <t>https://www.lennar.com/about/leadership/david-grove</t>
         </is>
       </c>
-      <c r="Y221" s="6" t="inlineStr"/>
+      <c r="Y221" s="6" t="inlineStr">
+        <is>
+          <t>2025-07-24 Dallas Morning News. The 10 biggest homebuilders in D-FW  https://www.dallasnews.com/business/real-estate/2025/07/24/list-who-are-the-10-biggest-homebuilders-in-d-fw/</t>
+        </is>
+      </c>
       <c r="Z221" s="6" t="inlineStr">
         <is>
           <t>(866) 314-4477</t>

</xml_diff>